<commit_message>
Daily slate 2026-06-28 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-26.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-26.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="E4" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F4" t="n">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="G4" t="n">
-        <v>46.2</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="E7" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F7" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G7" t="n">
-        <v>56.2</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="8">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E9" t="n">
         <v>98</v>
       </c>
       <c r="F9" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G9" t="n">
-        <v>67.09999999999999</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="10">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E10" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F10" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G10" t="n">
-        <v>59.8</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="11">
@@ -729,13 +729,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1319</v>
+        <v>1361</v>
       </c>
       <c r="E11" t="n">
-        <v>813</v>
+        <v>838</v>
       </c>
       <c r="F11" t="n">
-        <v>506</v>
+        <v>523</v>
       </c>
       <c r="G11" t="n">
         <v>61.6</v>
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="E12" t="n">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="F12" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G12" t="n">
-        <v>59.3</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="13">
@@ -787,16 +787,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G13" t="n">
-        <v>36.8</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="14">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>321</v>
+        <v>337</v>
       </c>
       <c r="E14" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F14" t="n">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="G14" t="n">
-        <v>21.5</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>487</v>
+        <v>516</v>
       </c>
       <c r="E15" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F15" t="n">
-        <v>396</v>
+        <v>423</v>
       </c>
       <c r="G15" t="n">
-        <v>18.7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -874,13 +874,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="E16" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F16" t="n">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="G16" t="n">
         <v>20.2</v>
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4787</v>
+        <v>4993</v>
       </c>
       <c r="E17" t="n">
-        <v>818</v>
+        <v>861</v>
       </c>
       <c r="F17" t="n">
-        <v>3969</v>
+        <v>4132</v>
       </c>
       <c r="G17" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
     </row>
   </sheetData>
@@ -1489,52 +1489,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>59.8</v>
+        <v>59.2</v>
       </c>
       <c r="C7" t="n">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D7" t="n">
         <v>61.6</v>
       </c>
       <c r="E7" t="n">
-        <v>1319</v>
+        <v>1361</v>
       </c>
       <c r="F7" t="n">
-        <v>59.3</v>
+        <v>60.1</v>
       </c>
       <c r="G7" t="n">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="H7" t="n">
-        <v>36.8</v>
+        <v>38.1</v>
       </c>
       <c r="I7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J7" t="n">
-        <v>21.5</v>
+        <v>20.8</v>
       </c>
       <c r="K7" t="n">
-        <v>321</v>
+        <v>337</v>
       </c>
       <c r="L7" t="n">
-        <v>18.7</v>
+        <v>18</v>
       </c>
       <c r="M7" t="n">
-        <v>487</v>
+        <v>516</v>
       </c>
       <c r="N7" t="n">
         <v>20.2</v>
       </c>
       <c r="O7" t="n">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="P7" t="n">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>4787</v>
+        <v>4993</v>
       </c>
       <c r="R7" t="n">
         <v>28.6</v>
@@ -1543,10 +1543,10 @@
         <v>7</v>
       </c>
       <c r="T7" t="n">
-        <v>46.2</v>
+        <v>45</v>
       </c>
       <c r="U7" t="n">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -1570,16 +1570,16 @@
         <v>2</v>
       </c>
       <c r="AD7" t="n">
-        <v>56.2</v>
+        <v>55.2</v>
       </c>
       <c r="AE7" t="n">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="AF7" t="n">
-        <v>67.09999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="AG7" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>